<commit_message>
Auto-allocation: groups fill themselves from a subject/class rule
Add group now leads with the teacher's name and the subject group she
takes: pick a subject column (EL, MA, ...), optionally a band value
('EL G2' or any-value) and/or a class filter ('1R' or '1R1,1R3'); code
and name are suggested automatically. On create, every matching student
is allocated instantly. New students arriving via school-file level
updates or the Add student dialog are auto-allocated to matching rule
groups too (restricted to just-added students, so manual removals are
never re-applied behind the admin's back). An explicit 'Auto-fill from
rule' button re-checks a group on demand; auto-fill only ever adds,
so hand adjustments always survive. Rules are stored in three new
Groups-sheet columns and shown in the groups table.

14 Node tests and 57 Playwright checks pass.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dce3QL9AfwtowDUpvwELb7
</commit_message>
<xml_diff>
--- a/sample/namelist.xlsx
+++ b/sample/namelist.xlsx
@@ -7335,12 +7335,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:G17"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7356,6 +7359,15 @@
       <c r="D1" t="str">
         <v>Teacher</v>
       </c>
+      <c r="E1" t="str">
+        <v>AutoSubject</v>
+      </c>
+      <c r="F1" t="str">
+        <v>AutoValue</v>
+      </c>
+      <c r="G1" t="str">
+        <v>AutoClasses</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -7370,6 +7382,15 @@
       <c r="D2" t="str">
         <v>Mrs Lim Bee Leng</v>
       </c>
+      <c r="E2" t="str">
+        <v>EL</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>1R1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -7384,6 +7405,15 @@
       <c r="D3" t="str">
         <v>Mr Rajesh Kumar</v>
       </c>
+      <c r="E3" t="str">
+        <v>MA</v>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v>1R1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -7398,6 +7428,15 @@
       <c r="D4" t="str">
         <v>Mr Daniel Tan</v>
       </c>
+      <c r="E4" t="str">
+        <v>EL</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>1R2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -7412,6 +7451,15 @@
       <c r="D5" t="str">
         <v>Mdm Halimah Yusof</v>
       </c>
+      <c r="E5" t="str">
+        <v>MA</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>1R2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -7426,6 +7474,15 @@
       <c r="D6" t="str">
         <v>Ms Nur Aisyah</v>
       </c>
+      <c r="E6" t="str">
+        <v>EL</v>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v>1R3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -7440,6 +7497,15 @@
       <c r="D7" t="str">
         <v>Ms Serene Goh</v>
       </c>
+      <c r="E7" t="str">
+        <v>MA</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v>1R3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -7454,6 +7520,15 @@
       <c r="D8" t="str">
         <v>Mrs Grace Chua</v>
       </c>
+      <c r="E8" t="str">
+        <v>EL</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v>1R4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -7468,6 +7543,15 @@
       <c r="D9" t="str">
         <v>Mr Alvin Ong</v>
       </c>
+      <c r="E9" t="str">
+        <v>MA</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>1R4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -7482,6 +7566,15 @@
       <c r="D10" t="str">
         <v>Mr Marcus Lee</v>
       </c>
+      <c r="E10" t="str">
+        <v>EL</v>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v>1R5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -7496,6 +7589,15 @@
       <c r="D11" t="str">
         <v>Mrs Doris Koh</v>
       </c>
+      <c r="E11" t="str">
+        <v>MA</v>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v>1R5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -7510,6 +7612,15 @@
       <c r="D12" t="str">
         <v>Mdm Sarimah Bakar</v>
       </c>
+      <c r="E12" t="str">
+        <v>EL</v>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v>1R6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -7524,6 +7635,15 @@
       <c r="D13" t="str">
         <v>Mr Wei Jie Chan</v>
       </c>
+      <c r="E13" t="str">
+        <v>MA</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v>1R6</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -7538,6 +7658,15 @@
       <c r="D14" t="str">
         <v>Dr Sarah Loh</v>
       </c>
+      <c r="E14" t="str">
+        <v>SCI</v>
+      </c>
+      <c r="F14" t="str">
+        <v>SCI G3</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -7552,6 +7681,15 @@
       <c r="D15" t="str">
         <v>Ms Priyanka Nair</v>
       </c>
+      <c r="E15" t="str">
+        <v>HIST</v>
+      </c>
+      <c r="F15" t="str">
+        <v>HIST G3</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -7566,6 +7704,15 @@
       <c r="D16" t="str">
         <v>Mr Kenneth Sim</v>
       </c>
+      <c r="E16" t="str">
+        <v>GEOG</v>
+      </c>
+      <c r="F16" t="str">
+        <v>GEOG G2</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -7580,10 +7727,19 @@
       <c r="D17" t="str">
         <v>Mrs Evelyn Phua</v>
       </c>
+      <c r="E17" t="str">
+        <v>LIT</v>
+      </c>
+      <c r="F17" t="str">
+        <v>LIT G3</v>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G17"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Keep each copy's folder to itself; subjects as a list; select-all
A copy of the app in a new folder reconnected to the ORIGINAL folder and saved
there, so the new folder's namelist.xlsx never changed and the copy looked
broken. Folder handles live in one IndexedDB for the whole file:// origin, so
they are now keyed to the folder the page itself was opened from: a copy starts
clean and asks which folder it should use, the original keeps its own, and the
start screen says so when a page's remembered folder is not the folder it sits
in.

Subjects become a list like teachers — New… adds one, later classes pick it
from the dropdown, Remove takes a wrong one off — stored in a Subjects sheet in
namelist.xlsx and seeded from whatever the classes already use.

Select-all where it was missing: one box takes every candidate shown in Group
members, and Tick all / Untick all work the class dialog's member list.
</commit_message>
<xml_diff>
--- a/sample/namelist.xlsx
+++ b/sample/namelist.xlsx
@@ -7,7 +7,8 @@
     <sheet name="Groups" sheetId="2" r:id="rId2"/>
     <sheet name="Memberships" sheetId="3" r:id="rId3"/>
     <sheet name="Teachers" sheetId="4" r:id="rId4"/>
-    <sheet name="Sources" sheetId="5" r:id="rId5"/>
+    <sheet name="Subjects" sheetId="5" r:id="rId5"/>
+    <sheet name="Sources" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -14546,6 +14547,55 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A7"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Subject</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>English Language</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Geography</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>History</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Literature</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Mathematics</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Science</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A7"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F2"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>

</xml_diff>